<commit_message>
Codici delle schede per modulo, schede in sola lettura nella pagina del modulo, PDF più leggibile
- Moduli con sigla (GEN, CMD, ELE, ...); schede della libreria numerate per modulo: GEN-01, GEN-02...
  La migrazione rinomina le schede NL esistenti e le loro copie nelle revisioni in bozza
  (le revisioni approvate restano com'erano). La sigla si importa dall'Excel (foglio Moduli).
- Pagina del modulo in amministrazione: elenco delle schede in sola lettura, senza il selettore
  che spostava schede da qualunque modulo.
- Valutazione dei rischi in PDF: riepilogo delle schede con esiti colorati, un modulo per pagina,
  testata per ogni scheda, dati in due colonne, valori della stima in grassetto con descrizione
  in grigio, misure raggruppate per tipo, rischio residuo in un riquadro; carattere più grande.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Confronto_librerie.xlsx
+++ b/dati/Confronto_librerie.xlsx
@@ -2362,7 +2362,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NL-001</t>
+          <t>GEN-01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>NL-002</t>
+          <t>GEN-02</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>NL-003</t>
+          <t>GEN-03</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>NL-004</t>
+          <t>GEN-04</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>NL-005</t>
+          <t>GEN-05</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>NL-006</t>
+          <t>GEN-06</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2608,7 +2608,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>NL-007</t>
+          <t>GEN-07</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>NL-008</t>
+          <t>GEN-08</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>NL-009</t>
+          <t>GEN-09</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2803,7 +2803,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>NL-010</t>
+          <t>GEN-10</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3083,7 +3083,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>NL-013</t>
+          <t>GEN-13</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>NL-011</t>
+          <t>GEN-11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>NL-012</t>
+          <t>GEN-12</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>NL-014</t>
+          <t>GEN-14</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>NL-015</t>
+          <t>GEN-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>NL-016</t>
+          <t>GEN-16</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3543,7 +3543,7 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>NL-078</t>
+          <t>PAS-01</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3578,7 +3578,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>NL-081</t>
+          <t>PAS-04</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3613,7 +3613,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>NL-079</t>
+          <t>PAS-02</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3648,7 +3648,7 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>NL-080</t>
+          <t>PAS-03</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3683,7 +3683,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>NL-017</t>
+          <t>CMD-01</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>NL-018</t>
+          <t>CMD-02</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>NL-019</t>
+          <t>CMD-03</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>NL-020</t>
+          <t>CMD-04</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>NL-021</t>
+          <t>CMD-05</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4046,7 +4046,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>NL-022</t>
+          <t>CMD-06</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>NL-023</t>
+          <t>CMD-07</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4198,7 +4198,7 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>NL-024</t>
+          <t>CMD-08</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>NL-025</t>
+          <t>CMD-09</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>NL-026</t>
+          <t>CMD-10</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>NL-032</t>
+          <t>CAB-06</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4444,7 +4444,7 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>NL-027</t>
+          <t>CAB-01</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>NL-028</t>
+          <t>CAB-02</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>NL-029</t>
+          <t>CAB-03</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>NL-030</t>
+          <t>CAB-04</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>NL-031</t>
+          <t>CAB-05</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -4803,7 +4803,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>NL-033</t>
+          <t>CAB-07</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4873,7 +4873,7 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>NL-036</t>
+          <t>TAV-03</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -5013,7 +5013,7 @@
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>NL-034</t>
+          <t>TAV-01</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5048,7 +5048,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>NL-037</t>
+          <t>TAV-04</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5118,7 +5118,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>NL-035</t>
+          <t>TAV-02</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -5153,7 +5153,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>NL-038</t>
+          <t>TAV-05</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5223,7 +5223,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>NL-039</t>
+          <t>ZSM-01</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -5258,7 +5258,7 @@
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>NL-043</t>
+          <t>ZSM-05</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -5293,7 +5293,7 @@
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>NL-040</t>
+          <t>ZSM-02</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5328,7 +5328,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>NL-041</t>
+          <t>ZSM-03</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -5363,7 +5363,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>NL-042</t>
+          <t>ZSM-04</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -5398,7 +5398,7 @@
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>NL-046</t>
+          <t>PAL-03</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -5433,7 +5433,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>NL-047</t>
+          <t>PAL-04</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>NL-044</t>
+          <t>PAL-01</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -5550,7 +5550,7 @@
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>NL-045</t>
+          <t>PAL-02</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -5585,7 +5585,7 @@
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>NL-051</t>
+          <t>ROB-04</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -5620,7 +5620,7 @@
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>NL-053</t>
+          <t>ROB-06</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -5725,7 +5725,7 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>NL-049</t>
+          <t>ROB-02</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -5760,7 +5760,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>NL-048</t>
+          <t>ROB-01</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -5795,7 +5795,7 @@
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>NL-050</t>
+          <t>ROB-03</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -5830,7 +5830,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>NL-052</t>
+          <t>ROB-05</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -5865,7 +5865,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>NL-054</t>
+          <t>ROB-07</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -5900,7 +5900,7 @@
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>NL-055</t>
+          <t>ROB-08</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -5935,7 +5935,7 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>NL-058</t>
+          <t>TRA-03</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>NL-057</t>
+          <t>TRA-02</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -6017,7 +6017,7 @@
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>NL-056</t>
+          <t>TRA-01</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -6052,7 +6052,7 @@
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>NL-059</t>
+          <t>TRA-04</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -6122,7 +6122,7 @@
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>NL-060</t>
+          <t>ZPU-01</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -6157,7 +6157,7 @@
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>NL-061</t>
+          <t>ZPU-02</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -6192,7 +6192,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>NL-062</t>
+          <t>ZPU-03</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -6227,7 +6227,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>NL-063</t>
+          <t>ZPU-04</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -6262,7 +6262,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>NL-066</t>
+          <t>LUC-03</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -6367,7 +6367,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>NL-065</t>
+          <t>LUC-02</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -6402,7 +6402,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>NL-064</t>
+          <t>LUC-01</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -6437,7 +6437,7 @@
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>NL-067</t>
+          <t>LUC-04</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -6472,7 +6472,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>NL-069</t>
+          <t>LUC-06</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -6542,7 +6542,7 @@
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>NL-068</t>
+          <t>LUC-05</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>NL-070</t>
+          <t>ELE-01</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -6620,7 +6620,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>NL-071</t>
+          <t>ELE-02</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>NL-073</t>
+          <t>ELE-04</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -6737,7 +6737,7 @@
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>NL-072</t>
+          <t>ELE-03</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -6772,7 +6772,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
-          <t>NL-076</t>
+          <t>PNE-03</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>NL-074</t>
+          <t>PNE-01</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -6850,7 +6850,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>NL-077</t>
+          <t>PNE-04</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -6885,7 +6885,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>NL-075</t>
+          <t>PNE-02</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>NL-082</t>
+          <t>INF-01</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>NL-083</t>
+          <t>INF-02</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -7061,7 +7061,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>NL-084</t>
+          <t>INF-03</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>NL-085</t>
+          <t>INF-04</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>NL-086</t>
+          <t>INF-05</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>NL-087</t>
+          <t>INF-06</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -7256,7 +7256,7 @@
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>NL-088</t>
+          <t>INF-07</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">

</xml_diff>

<commit_message>
Codici delle schede SIGLA-RESS-indice (es. TAV-1.3.8.2-1)
L'indice parte da 1 per ogni coppia modulo/RESS e distingue le schede dello stesso requisito.
La migrazione converte i codici SIGLA-NN della libreria e delle revisioni in bozza; le schede
modello si ordinano per modulo e requisito come quelle dell'analisi.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Confronto_librerie.xlsx
+++ b/dati/Confronto_librerie.xlsx
@@ -2362,7 +2362,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>GEN-01</t>
+          <t>GEN-1.1.1-1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>GEN-02</t>
+          <t>GEN-1.1.2-1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>GEN-03</t>
+          <t>GEN-1.1.3-1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>GEN-04</t>
+          <t>GEN-1.1.4-1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GEN-05</t>
+          <t>GEN-1.1.5-1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GEN-06</t>
+          <t>GEN-1.1.6-1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2608,7 +2608,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>GEN-07</t>
+          <t>GEN-1.1.7-1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>GEN-08</t>
+          <t>GEN-1.3.1-1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>GEN-09</t>
+          <t>GEN-1.3.4-1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2803,7 +2803,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>GEN-10</t>
+          <t>GEN-1.3.5-1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3083,7 +3083,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>GEN-13</t>
+          <t>GEN-1.5.15-1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>GEN-11</t>
+          <t>GEN-1.5.4-1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>GEN-12</t>
+          <t>GEN-1.5.8-1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>GEN-14</t>
+          <t>GEN-1.6.1-1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>GEN-15</t>
+          <t>GEN-1.6.2-1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>GEN-16</t>
+          <t>GEN-1.6.4-1</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3543,7 +3543,7 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PAS-01</t>
+          <t>PAS-1.5.13-1</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3578,7 +3578,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PAS-04</t>
+          <t>PAS-1.5.15-1</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3613,7 +3613,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PAS-02</t>
+          <t>PAS-1.5.3-1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3648,7 +3648,7 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PAS-03</t>
+          <t>PAS-1.6.1-1</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3683,7 +3683,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CMD-01</t>
+          <t>CMD-1.1.9-1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CMD-02</t>
+          <t>CMD-1.2.1-1</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CMD-03</t>
+          <t>CMD-1.2.2-1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CMD-04</t>
+          <t>CMD-1.2.3-1</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CMD-05</t>
+          <t>CMD-1.2.4.1-1</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4046,7 +4046,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>CMD-06</t>
+          <t>CMD-1.2.4.2-1</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>CMD-07</t>
+          <t>CMD-1.2.4.3-1</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4198,7 +4198,7 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>CMD-08</t>
+          <t>CMD-1.2.4.4-1</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>CMD-09</t>
+          <t>CMD-1.2.5-1</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>CMD-10</t>
+          <t>CMD-1.2.6-1</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>CAB-06</t>
+          <t>CAB-1.3.3-1</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4444,7 +4444,7 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>CAB-01</t>
+          <t>CAB-1.3.7-1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>CAB-02</t>
+          <t>CAB-1.4.1-1</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>CAB-03</t>
+          <t>CAB-1.4.2.1-1</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CAB-04</t>
+          <t>CAB-1.4.2.2-1</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>CAB-05</t>
+          <t>CAB-1.4.3-1</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -4803,7 +4803,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>CAB-07</t>
+          <t>CAB-1.5.14-1</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4873,7 +4873,7 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>TAV-03</t>
+          <t>TAV-1.1.6-1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -5013,7 +5013,7 @@
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TAV-01</t>
+          <t>TAV-1.3.8.2-1</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5048,7 +5048,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>TAV-04</t>
+          <t>TAV-1.3.9-1</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5118,7 +5118,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>TAV-02</t>
+          <t>TAV-1.4.3-1</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -5153,7 +5153,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>TAV-05</t>
+          <t>TAV-1.5.5-1</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5223,7 +5223,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>ZSM-01</t>
+          <t>ZSM-1.5.13-1</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -5258,7 +5258,7 @@
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>ZSM-05</t>
+          <t>ZSM-1.5.2-1</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -5293,7 +5293,7 @@
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>ZSM-02</t>
+          <t>ZSM-1.5.6-1</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5328,7 +5328,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>ZSM-03</t>
+          <t>ZSM-1.5.7-1</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -5363,7 +5363,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>ZSM-04</t>
+          <t>ZSM-1.6.5-1</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -5398,7 +5398,7 @@
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>PAL-03</t>
+          <t>PAL-1.1.6-1</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -5433,7 +5433,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>PAL-04</t>
+          <t>PAL-1.3.3-1</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>PAL-1.3.7-1</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -5550,7 +5550,7 @@
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>PAL-1.4.3-1</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -5585,7 +5585,7 @@
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>ROB-04</t>
+          <t>ROB-1.3.2-1</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -5620,7 +5620,7 @@
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>ROB-06</t>
+          <t>ROB-1.3.6-1</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -5725,7 +5725,7 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>ROB-02</t>
+          <t>ROB-1.3.8.1-1</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -5760,7 +5760,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>ROB-01</t>
+          <t>ROB-1.3.8.2-1</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -5795,7 +5795,7 @@
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>ROB-03</t>
+          <t>ROB-1.3.8.2-2</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -5830,7 +5830,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>ROB-05</t>
+          <t>ROB-1.3.9-1</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -5865,7 +5865,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>ROB-07</t>
+          <t>ROB-1.5.5-1</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -5900,7 +5900,7 @@
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>ROB-08</t>
+          <t>ROB-1.6.4-1</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -5935,7 +5935,7 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>TRA-03</t>
+          <t>TRA-1.2.4.3-1</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>TRA-02</t>
+          <t>TRA-1.3.7-1</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -6017,7 +6017,7 @@
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>TRA-01</t>
+          <t>TRA-1.3.8.1-1</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -6052,7 +6052,7 @@
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>TRA-04</t>
+          <t>TRA-1.5.5-1</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -6122,7 +6122,7 @@
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>ZPU-01</t>
+          <t>ZPU-1.5.13-1</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -6157,7 +6157,7 @@
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>ZPU-02</t>
+          <t>ZPU-1.5.6-1</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -6192,7 +6192,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>ZPU-03</t>
+          <t>ZPU-1.5.7-1</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -6227,7 +6227,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>ZPU-04</t>
+          <t>ZPU-1.6.5-1</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -6262,7 +6262,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>LUC-03</t>
+          <t>LUC-1.3.2-1</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -6367,7 +6367,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>LUC-02</t>
+          <t>LUC-1.3.8.1-1</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -6402,7 +6402,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>LUC-01</t>
+          <t>LUC-1.3.8.2-1</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -6437,7 +6437,7 @@
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>LUC-04</t>
+          <t>LUC-1.3.9-1</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -6472,7 +6472,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>LUC-06</t>
+          <t>LUC-1.5.5-1</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -6542,7 +6542,7 @@
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>LUC-05</t>
+          <t>LUC-1.6.4-1</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>ELE-1.5.1-1</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -6620,7 +6620,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>ELE-02</t>
+          <t>ELE-1.5.1-2</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>ELE-04</t>
+          <t>ELE-1.5.6-1</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -6737,7 +6737,7 @@
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>ELE-03</t>
+          <t>ELE-1.6.3-1</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -6772,7 +6772,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
-          <t>PNE-03</t>
+          <t>PNE-1.2.6-1</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>PNE-01</t>
+          <t>PNE-1.5.3-1</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -6850,7 +6850,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>PNE-04</t>
+          <t>PNE-1.5.8-1</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -6885,7 +6885,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>PNE-02</t>
+          <t>PNE-1.6.3-1</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>INF-01</t>
+          <t>INF-1.7.1.1-1</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>INF-02</t>
+          <t>INF-1.7.1.2-1</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -7061,7 +7061,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>INF-03</t>
+          <t>INF-1.7.2-1</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>INF-04</t>
+          <t>INF-1.7.3-1</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>INF-05</t>
+          <t>INF-1.7.4.1-1</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>INF-06</t>
+          <t>INF-1.7.4.2-1</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -7256,7 +7256,7 @@
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>INF-07</t>
+          <t>INF-1.7.4.3-1</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">

</xml_diff>

<commit_message>
Ritorno ai codici progressivi per modulo (GEN-01), ordine per RESS, codice a destra nel PDF
- Codici delle schede SIGLA-NN: la migrazione 0013 ripristina esattamente i codici precedenti
  della libreria NL e delle copie in bozza; le schede nuove prendono il numero successivo nel
  modulo (libreria e schede aggiunte nell'analisi), che cambia solo se cambia il modulo.
- L'ordine di visualizzazione resta quello del requisito RESS.
- PDF: requisito a sinistra e codice della scheda a destra (testate, riepilogo, schede scartate,
  rischi residui).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Confronto_librerie.xlsx
+++ b/dati/Confronto_librerie.xlsx
@@ -2362,7 +2362,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>GEN-1.1.1-1</t>
+          <t>GEN-01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>GEN-1.1.2-1</t>
+          <t>GEN-02</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>GEN-1.1.3-1</t>
+          <t>GEN-03</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>GEN-1.1.4-1</t>
+          <t>GEN-04</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GEN-1.1.5-1</t>
+          <t>GEN-05</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GEN-1.1.6-1</t>
+          <t>GEN-06</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2608,7 +2608,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>GEN-1.1.7-1</t>
+          <t>GEN-07</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>GEN-1.3.1-1</t>
+          <t>GEN-08</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>GEN-1.3.4-1</t>
+          <t>GEN-09</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2803,7 +2803,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>GEN-1.3.5-1</t>
+          <t>GEN-10</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3083,7 +3083,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>GEN-1.5.15-1</t>
+          <t>GEN-13</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>GEN-1.5.4-1</t>
+          <t>GEN-11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>GEN-1.5.8-1</t>
+          <t>GEN-12</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>GEN-1.6.1-1</t>
+          <t>GEN-14</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>GEN-1.6.2-1</t>
+          <t>GEN-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>GEN-1.6.4-1</t>
+          <t>GEN-16</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3543,7 +3543,7 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PAS-1.5.13-1</t>
+          <t>PAS-01</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3578,7 +3578,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PAS-1.5.15-1</t>
+          <t>PAS-04</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3613,7 +3613,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PAS-1.5.3-1</t>
+          <t>PAS-02</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3648,7 +3648,7 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PAS-1.6.1-1</t>
+          <t>PAS-03</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3683,7 +3683,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CMD-1.1.9-1</t>
+          <t>CMD-01</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CMD-1.2.1-1</t>
+          <t>CMD-02</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CMD-1.2.2-1</t>
+          <t>CMD-03</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CMD-1.2.3-1</t>
+          <t>CMD-04</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CMD-1.2.4.1-1</t>
+          <t>CMD-05</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4046,7 +4046,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>CMD-1.2.4.2-1</t>
+          <t>CMD-06</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>CMD-1.2.4.3-1</t>
+          <t>CMD-07</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4198,7 +4198,7 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>CMD-1.2.4.4-1</t>
+          <t>CMD-08</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>CMD-1.2.5-1</t>
+          <t>CMD-09</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>CMD-1.2.6-1</t>
+          <t>CMD-10</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>CAB-1.3.3-1</t>
+          <t>CAB-06</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4444,7 +4444,7 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>CAB-1.3.7-1</t>
+          <t>CAB-01</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>CAB-1.4.1-1</t>
+          <t>CAB-02</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>CAB-1.4.2.1-1</t>
+          <t>CAB-03</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CAB-1.4.2.2-1</t>
+          <t>CAB-04</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>CAB-1.4.3-1</t>
+          <t>CAB-05</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -4803,7 +4803,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>CAB-1.5.14-1</t>
+          <t>CAB-07</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4873,7 +4873,7 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>TAV-1.1.6-1</t>
+          <t>TAV-03</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -5013,7 +5013,7 @@
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TAV-1.3.8.2-1</t>
+          <t>TAV-01</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5048,7 +5048,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>TAV-1.3.9-1</t>
+          <t>TAV-04</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5118,7 +5118,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>TAV-1.4.3-1</t>
+          <t>TAV-02</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -5153,7 +5153,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>TAV-1.5.5-1</t>
+          <t>TAV-05</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5223,7 +5223,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>ZSM-1.5.13-1</t>
+          <t>ZSM-01</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -5258,7 +5258,7 @@
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>ZSM-1.5.2-1</t>
+          <t>ZSM-05</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -5293,7 +5293,7 @@
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>ZSM-1.5.6-1</t>
+          <t>ZSM-02</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5328,7 +5328,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>ZSM-1.5.7-1</t>
+          <t>ZSM-03</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -5363,7 +5363,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>ZSM-1.6.5-1</t>
+          <t>ZSM-04</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -5398,7 +5398,7 @@
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>PAL-1.1.6-1</t>
+          <t>PAL-03</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -5433,7 +5433,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>PAL-1.3.3-1</t>
+          <t>PAL-04</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>PAL-1.3.7-1</t>
+          <t>PAL-01</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -5550,7 +5550,7 @@
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>PAL-1.4.3-1</t>
+          <t>PAL-02</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -5585,7 +5585,7 @@
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>ROB-1.3.2-1</t>
+          <t>ROB-04</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -5620,7 +5620,7 @@
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>ROB-1.3.6-1</t>
+          <t>ROB-06</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -5725,7 +5725,7 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>ROB-1.3.8.1-1</t>
+          <t>ROB-02</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -5760,7 +5760,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>ROB-1.3.8.2-1</t>
+          <t>ROB-01</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -5795,7 +5795,7 @@
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>ROB-1.3.8.2-2</t>
+          <t>ROB-03</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -5830,7 +5830,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>ROB-1.3.9-1</t>
+          <t>ROB-05</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -5865,7 +5865,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>ROB-1.5.5-1</t>
+          <t>ROB-07</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -5900,7 +5900,7 @@
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>ROB-1.6.4-1</t>
+          <t>ROB-08</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -5935,7 +5935,7 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>TRA-1.2.4.3-1</t>
+          <t>TRA-03</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>TRA-1.3.7-1</t>
+          <t>TRA-02</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -6017,7 +6017,7 @@
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>TRA-1.3.8.1-1</t>
+          <t>TRA-01</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -6052,7 +6052,7 @@
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>TRA-1.5.5-1</t>
+          <t>TRA-04</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -6122,7 +6122,7 @@
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>ZPU-1.5.13-1</t>
+          <t>ZPU-01</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -6157,7 +6157,7 @@
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>ZPU-1.5.6-1</t>
+          <t>ZPU-02</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -6192,7 +6192,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>ZPU-1.5.7-1</t>
+          <t>ZPU-03</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -6227,7 +6227,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>ZPU-1.6.5-1</t>
+          <t>ZPU-04</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -6262,7 +6262,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>LUC-1.3.2-1</t>
+          <t>LUC-03</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -6367,7 +6367,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>LUC-1.3.8.1-1</t>
+          <t>LUC-02</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -6402,7 +6402,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>LUC-1.3.8.2-1</t>
+          <t>LUC-01</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -6437,7 +6437,7 @@
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>LUC-1.3.9-1</t>
+          <t>LUC-04</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -6472,7 +6472,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>LUC-1.5.5-1</t>
+          <t>LUC-06</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -6542,7 +6542,7 @@
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>LUC-1.6.4-1</t>
+          <t>LUC-05</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>ELE-1.5.1-1</t>
+          <t>ELE-01</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -6620,7 +6620,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>ELE-1.5.1-2</t>
+          <t>ELE-02</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>ELE-1.5.6-1</t>
+          <t>ELE-04</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -6737,7 +6737,7 @@
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>ELE-1.6.3-1</t>
+          <t>ELE-03</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -6772,7 +6772,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
-          <t>PNE-1.2.6-1</t>
+          <t>PNE-03</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>PNE-1.5.3-1</t>
+          <t>PNE-01</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -6850,7 +6850,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>PNE-1.5.8-1</t>
+          <t>PNE-04</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -6885,7 +6885,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>PNE-1.6.3-1</t>
+          <t>PNE-02</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>INF-1.7.1.1-1</t>
+          <t>INF-01</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>INF-1.7.1.2-1</t>
+          <t>INF-02</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -7061,7 +7061,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>INF-1.7.2-1</t>
+          <t>INF-03</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>INF-1.7.3-1</t>
+          <t>INF-04</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>INF-1.7.4.1-1</t>
+          <t>INF-05</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>INF-1.7.4.2-1</t>
+          <t>INF-06</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -7256,7 +7256,7 @@
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>INF-1.7.4.3-1</t>
+          <t>INF-07</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">

</xml_diff>